<commit_message>
Refactor index.html and update asset versioning; enhance CSV and XLSX export functionality with filtering and pagination; improve test coverage for data processing and layout consistency.
</commit_message>
<xml_diff>
--- a/exemplo-ncm-cst-cclasstrib.xlsx
+++ b/exemplo-ncm-cst-cclasstrib.xlsx
@@ -48,16 +48,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="58" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
     <col min="9" max="9" width="5" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="8" customWidth="1"/>
+    <col min="10" max="10" width="5" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="12" max="12" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -68,50 +69,55 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Descrição NCM</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">CST</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">cClassTrib</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Descrição</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Descrição CClassTrib</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Tipo alíq.</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Redução</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">CP</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">EC</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">DF-e</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Anexos</t>
         </is>
@@ -125,32 +131,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Legumes de vagem, mesmo com vagem, frescos ou refrigerados. — Feijões (Vigna spp., Phaseolus spp.)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t xml:space="preserve">200014</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos produtos hortícolas, frutas e ovos (Anexo XV)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% · 100%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 100% · IBS 100%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -165,10 +171,15 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, DUIMP</t>
         </is>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>134</v>
       </c>
     </row>
@@ -180,32 +191,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Legumes de vagem, mesmo com vagem, frescos ou refrigerados. — Feijões (Vigna spp., Phaseolus spp.)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t xml:space="preserve">200034</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos alimentos destinados ao consumo humano (Anexo VII)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -220,10 +231,15 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, DUIMP</t>
         </is>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>446</v>
       </c>
     </row>
@@ -235,32 +251,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Legumes de vagem, mesmo com vagem, frescos ou refrigerados. — Feijões (Vigna spp., Phaseolus spp.)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t xml:space="preserve">200038</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -275,10 +291,15 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>1189</v>
       </c>
     </row>
@@ -290,32 +311,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Legumes de vagem, mesmo com vagem, frescos ou refrigerados. — Feijões (Vigna spp., Phaseolus spp.)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t xml:space="preserve">515</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">515001</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t xml:space="preserve">Operações, sujeitas a diferimento, com insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -330,10 +351,15 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>1189</v>
       </c>
     </row>
@@ -345,32 +371,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Arroz. — Arroz descascado (arroz cargo ou castanho) — Parboilizado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t xml:space="preserve">200003</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t xml:space="preserve">Vendas de produtos destinados à alimentação humana (Anexo I)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% · 100%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 100% · IBS 100%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -385,10 +411,15 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, DUIMP</t>
         </is>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>361</v>
       </c>
     </row>
@@ -400,32 +431,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Arroz. — Arroz descascado (arroz cargo ou castanho) — Parboilizado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t xml:space="preserve">200034</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos alimentos destinados ao consumo humano (Anexo VII)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -440,10 +471,15 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, DUIMP</t>
         </is>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>446</v>
       </c>
     </row>
@@ -455,32 +491,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Arroz. — Arroz descascado (arroz cargo ou castanho) — Parboilizado</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t xml:space="preserve">200038</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -495,10 +531,15 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>1189</v>
       </c>
     </row>
@@ -510,32 +551,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Arroz. — Arroz descascado (arroz cargo ou castanho) — Parboilizado</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t xml:space="preserve">515</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">515001</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t xml:space="preserve">Operações, sujeitas a diferimento, com insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -550,10 +591,15 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>1189</v>
       </c>
     </row>
@@ -565,32 +611,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho. — Outros — Outros — Outros</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t xml:space="preserve">200005</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento de dispositivos médicos para órgãos da administração pública e entidades de saúde imunes (Anexo IV)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% · 100%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 100% · IBS 100%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -605,10 +651,15 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>144</v>
       </c>
     </row>
@@ -620,32 +671,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho. — Outros — Outros — Outros</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t xml:space="preserve">200030</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda dos dispositivos médicos  (Anexo IV)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -660,10 +711,15 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>144</v>
       </c>
     </row>
@@ -675,32 +731,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho. — Outros — Outros — Outros</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t xml:space="preserve">200032</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos medicamentos registrados na Anvisa ou produzidos por farmácias de manipulação, ressalvados os medicamentos sujeitos à alíquota zero</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -715,10 +771,15 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, DIR, DUIMP</t>
         </is>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>382</v>
       </c>
     </row>
@@ -730,32 +791,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho. — Outros — Outros — Outros</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t xml:space="preserve">200038</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento dos insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -770,10 +831,15 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>1189</v>
       </c>
     </row>
@@ -785,32 +851,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t xml:space="preserve">Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho. — Outros — Outros — Outros</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t xml:space="preserve">515</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t xml:space="preserve">515001</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">Operações, sujeitas a diferimento, com insumos agropecuários e aquícolas (Anexo IX)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -825,10 +891,15 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>1189</v>
       </c>
     </row>
@@ -838,20 +909,57 @@
           <t xml:space="preserve">01012100</t>
         </is>
       </c>
-      <c r="B15"/>
-      <c r="C15"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cavalos, asininos e muares, vivos. — Cavalos: — Reprodutores de raça pura</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cavalos, asininos e muares, vivos. — Cavalos: — Reprodutores de raça pura</t>
-        </is>
-      </c>
-      <c r="E15"/>
-      <c r="F15"/>
-      <c r="G15"/>
-      <c r="H15"/>
-      <c r="I15"/>
-      <c r="J15"/>
-      <c r="K15"/>
+          <t xml:space="preserve">000001</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Situações tributadas integralmente pelo IBS e CBS.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 — Padrão</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFe, NFCe, CTe, CTe-OS, BPe, BPe-TA, NF3e, NFCom, NFSe, NFGAS, NFAg, DIR, DUIMP</t>
+        </is>
+      </c>
+      <c r="L15"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -861,32 +969,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Aparelhos e equipamentos para laboratórios fotográficos ou cinematográficos, não especificados nem compreendidos noutras posições do presente Capítulo; negatoscópios; telas para projeção. — Instrumentos e aparelhos para medicina, cirurgia, odontologia e veterinária, incluindo os aparelhos para cintilografia e outros aparelhos eletromédicos, bem como os aparelhos para testes visuais. — Seringas, agulhas, cateteres, cânulas e instrumentos semelhantes: — Outros — Agulhas</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t xml:space="preserve">200005</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t xml:space="preserve">Fornecimento de dispositivos médicos para órgãos da administração pública e entidades de saúde imunes (Anexo IV)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% · 100%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 100% · IBS 100%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -901,10 +1009,15 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>144</v>
       </c>
     </row>
@@ -916,32 +1029,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">Aparelhos e equipamentos para laboratórios fotográficos ou cinematográficos, não especificados nem compreendidos noutras posições do presente Capítulo; negatoscópios; telas para projeção. — Instrumentos e aparelhos para medicina, cirurgia, odontologia e veterinária, incluindo os aparelhos para cintilografia e outros aparelhos eletromédicos, bem como os aparelhos para testes visuais. — Seringas, agulhas, cateteres, cânulas e instrumentos semelhantes: — Outros — Agulhas</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t xml:space="preserve">200</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t xml:space="preserve">200030</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda dos dispositivos médicos  (Anexo IV)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 — Padrão</t>
-        </is>
-      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">60% · 60%</t>
+          <t xml:space="preserve">2 — Padrão</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">CBS 60% · IBS 60%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -956,10 +1069,15 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
           <t xml:space="preserve">NFe, NFCe, NFSe, DUIMP</t>
         </is>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>144</v>
       </c>
     </row>

</xml_diff>